<commit_message>
data: update 7 sources
</commit_message>
<xml_diff>
--- a/xlsx/CPE.xlsx
+++ b/xlsx/CPE.xlsx
@@ -123,8 +123,7 @@
 3. Allegro (A major)</t>
   </si>
   <si>
-    <t>Aussi version pour flûte traversière et cordes (Wq 168/H 438);
-violoncelle et cordes (Wq 172/H 439)</t>
+    <t>Aussi version pour flûte traversière et cordes (Wq 168/H 438); violoncelle et cordes (Wq 172/H 439)</t>
   </si>
   <si>
     <t>Wq. 168</t>
@@ -144,8 +143,7 @@
     <t>Transverse Flute, 2 Violins, Viola, Basso</t>
   </si>
   <si>
-    <t>Aussi version pour clavecin et cordes (Wq 29/H 437);
-violoncelle et cordes (Wq 172/H 439)</t>
+    <t>Aussi version pour clavecin et cordes (Wq 29/H 437); violoncelle et cordes (Wq 172/H 439)</t>
   </si>
   <si>
     <t>Wq. 172</t>
@@ -12502,6 +12500,10 @@
       <c r="C106" s="3" t="s">
         <v>381</v>
       </c>
+      <c r="D106" s="4" t="str">
+        <f t="shared" ref="D106:D112" si="0">E106&amp;" in "&amp;F106</f>
+        <v>Duet in A minor</v>
+      </c>
       <c r="E106" s="5" t="s">
         <v>382</v>
       </c>
@@ -12522,6 +12524,10 @@
       <c r="C107" s="3" t="s">
         <v>385</v>
       </c>
+      <c r="D107" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>Duet in B-flat major</v>
+      </c>
       <c r="E107" s="5" t="s">
         <v>382</v>
       </c>
@@ -12539,6 +12545,10 @@
       <c r="C108" s="3" t="s">
         <v>387</v>
       </c>
+      <c r="D108" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>Duet in C major</v>
+      </c>
       <c r="E108" s="5" t="s">
         <v>382</v>
       </c>
@@ -12559,6 +12569,10 @@
       <c r="C109" s="3" t="s">
         <v>390</v>
       </c>
+      <c r="D109" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>Duet in D minor</v>
+      </c>
       <c r="E109" s="5" t="s">
         <v>382</v>
       </c>
@@ -12579,6 +12593,10 @@
       <c r="C110" s="3" t="s">
         <v>393</v>
       </c>
+      <c r="D110" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>Duet in E minor</v>
+      </c>
       <c r="E110" s="5" t="s">
         <v>382</v>
       </c>
@@ -12599,6 +12617,10 @@
       <c r="C111" s="3" t="s">
         <v>396</v>
       </c>
+      <c r="D111" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>Duet in E-flat major</v>
+      </c>
       <c r="E111" s="5" t="s">
         <v>382</v>
       </c>
@@ -12619,6 +12641,10 @@
       <c r="C112" s="3" t="s">
         <v>398</v>
       </c>
+      <c r="D112" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>Duet in F major</v>
+      </c>
       <c r="E112" s="5" t="s">
         <v>382</v>
       </c>
@@ -12653,6 +12679,10 @@
       <c r="C114" s="3" t="s">
         <v>401</v>
       </c>
+      <c r="D114" s="4" t="str">
+        <f t="shared" ref="D114:D119" si="1">E114&amp;" in "&amp;F114</f>
+        <v>Fantasia in A major</v>
+      </c>
       <c r="E114" s="5" t="s">
         <v>402</v>
       </c>
@@ -12673,6 +12703,10 @@
       <c r="C115" s="3" t="s">
         <v>404</v>
       </c>
+      <c r="D115" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fantasia in B-flat major</v>
+      </c>
       <c r="E115" s="5" t="s">
         <v>402</v>
       </c>
@@ -12693,6 +12727,10 @@
       <c r="C116" s="3" t="s">
         <v>404</v>
       </c>
+      <c r="D116" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fantasia in B-flat major</v>
+      </c>
       <c r="E116" s="5" t="s">
         <v>402</v>
       </c>
@@ -12713,6 +12751,10 @@
       <c r="C117" s="3" t="s">
         <v>407</v>
       </c>
+      <c r="D117" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fantasia in B-flat major</v>
+      </c>
       <c r="E117" s="5" t="s">
         <v>402</v>
       </c>
@@ -12733,6 +12775,10 @@
       <c r="C118" s="3" t="s">
         <v>409</v>
       </c>
+      <c r="D118" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fantasia in C major</v>
+      </c>
       <c r="E118" s="5" t="s">
         <v>402</v>
       </c>
@@ -12753,6 +12799,10 @@
       <c r="C119" s="3" t="s">
         <v>411</v>
       </c>
+      <c r="D119" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fantasia in C major</v>
+      </c>
       <c r="E119" s="5" t="s">
         <v>402</v>
       </c>
@@ -12796,6 +12846,10 @@
       <c r="C121" s="3" t="s">
         <v>416</v>
       </c>
+      <c r="D121" s="4" t="str">
+        <f t="shared" ref="D121:D133" si="2">E121&amp;" in "&amp;F121</f>
+        <v>Fantasia in D major</v>
+      </c>
       <c r="E121" s="5" t="s">
         <v>402</v>
       </c>
@@ -12816,6 +12870,10 @@
       <c r="C122" s="3" t="s">
         <v>416</v>
       </c>
+      <c r="D122" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in D major</v>
+      </c>
       <c r="E122" s="5" t="s">
         <v>402</v>
       </c>
@@ -12836,6 +12894,10 @@
       <c r="C123" s="3" t="s">
         <v>419</v>
       </c>
+      <c r="D123" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in D major</v>
+      </c>
       <c r="E123" s="5" t="s">
         <v>402</v>
       </c>
@@ -12856,6 +12918,10 @@
       <c r="C124" s="3" t="s">
         <v>421</v>
       </c>
+      <c r="D124" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in D minor</v>
+      </c>
       <c r="E124" s="5" t="s">
         <v>402</v>
       </c>
@@ -12876,6 +12942,10 @@
       <c r="C125" s="3" t="s">
         <v>421</v>
       </c>
+      <c r="D125" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in D minor</v>
+      </c>
       <c r="E125" s="5" t="s">
         <v>402</v>
       </c>
@@ -12896,6 +12966,10 @@
       <c r="C126" s="3" t="s">
         <v>424</v>
       </c>
+      <c r="D126" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in D minor</v>
+      </c>
       <c r="E126" s="5" t="s">
         <v>402</v>
       </c>
@@ -12916,6 +12990,10 @@
       <c r="C127" s="3" t="s">
         <v>426</v>
       </c>
+      <c r="D127" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in D minor</v>
+      </c>
       <c r="E127" s="5" t="s">
         <v>402</v>
       </c>
@@ -12936,6 +13014,10 @@
       <c r="C128" s="3" t="s">
         <v>426</v>
       </c>
+      <c r="D128" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in D minor</v>
+      </c>
       <c r="E128" s="5" t="s">
         <v>402</v>
       </c>
@@ -12956,6 +13038,10 @@
       <c r="C129" s="3" t="s">
         <v>429</v>
       </c>
+      <c r="D129" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in E-flat major</v>
+      </c>
       <c r="E129" s="5" t="s">
         <v>402</v>
       </c>
@@ -12976,6 +13062,10 @@
       <c r="C130" s="3" t="s">
         <v>431</v>
       </c>
+      <c r="D130" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in F major</v>
+      </c>
       <c r="E130" s="5" t="s">
         <v>402</v>
       </c>
@@ -12996,6 +13086,10 @@
       <c r="C131" s="3" t="s">
         <v>431</v>
       </c>
+      <c r="D131" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in F major</v>
+      </c>
       <c r="E131" s="5" t="s">
         <v>402</v>
       </c>
@@ -13016,6 +13110,10 @@
       <c r="C132" s="3" t="s">
         <v>434</v>
       </c>
+      <c r="D132" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in F major</v>
+      </c>
       <c r="E132" s="5" t="s">
         <v>402</v>
       </c>
@@ -13036,6 +13134,10 @@
       <c r="C133" s="3" t="s">
         <v>436</v>
       </c>
+      <c r="D133" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Fantasia in F-sharp minor</v>
+      </c>
       <c r="E133" s="5" t="s">
         <v>402</v>
       </c>
@@ -13079,6 +13181,10 @@
       <c r="C135" s="3" t="s">
         <v>443</v>
       </c>
+      <c r="D135" s="4" t="str">
+        <f>E135&amp;" in "&amp;F135</f>
+        <v>Fantasia in G major</v>
+      </c>
       <c r="E135" s="5" t="s">
         <v>402</v>
       </c>
@@ -13099,6 +13205,10 @@
       <c r="C136" s="3" t="s">
         <v>445</v>
       </c>
+      <c r="D136" s="4" t="str">
+        <f>E136&amp;" in "&amp;F136</f>
+        <v>Fantasia in G minor</v>
+      </c>
       <c r="E136" s="5" t="s">
         <v>402</v>
       </c>
@@ -16422,6 +16532,10 @@
       <c r="C299" s="3" t="s">
         <v>871</v>
       </c>
+      <c r="D299" s="4" t="str">
+        <f t="shared" ref="D299:D311" si="3">E299&amp;" in "&amp;F299</f>
+        <v>March in C major</v>
+      </c>
       <c r="E299" s="5" t="s">
         <v>872</v>
       </c>
@@ -16465,6 +16579,10 @@
       <c r="C301" s="3" t="s">
         <v>879</v>
       </c>
+      <c r="D301" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in D major</v>
+      </c>
       <c r="E301" s="5" t="s">
         <v>872</v>
       </c>
@@ -16485,6 +16603,10 @@
       <c r="C302" s="3" t="s">
         <v>881</v>
       </c>
+      <c r="D302" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in D major</v>
+      </c>
       <c r="E302" s="5" t="s">
         <v>872</v>
       </c>
@@ -16505,6 +16627,10 @@
       <c r="C303" s="3" t="s">
         <v>883</v>
       </c>
+      <c r="D303" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in D major</v>
+      </c>
       <c r="E303" s="5" t="s">
         <v>872</v>
       </c>
@@ -16522,6 +16648,10 @@
       <c r="C304" s="3" t="s">
         <v>885</v>
       </c>
+      <c r="D304" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in D major</v>
+      </c>
       <c r="E304" s="5" t="s">
         <v>872</v>
       </c>
@@ -16539,6 +16669,10 @@
       <c r="C305" s="3" t="s">
         <v>887</v>
       </c>
+      <c r="D305" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in D major</v>
+      </c>
       <c r="E305" s="5" t="s">
         <v>872</v>
       </c>
@@ -16559,6 +16693,10 @@
       <c r="C306" s="3" t="s">
         <v>890</v>
       </c>
+      <c r="D306" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in E-flat major</v>
+      </c>
       <c r="E306" s="5" t="s">
         <v>872</v>
       </c>
@@ -16579,6 +16717,10 @@
       <c r="C307" s="3" t="s">
         <v>892</v>
       </c>
+      <c r="D307" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in F major</v>
+      </c>
       <c r="E307" s="5" t="s">
         <v>872</v>
       </c>
@@ -16599,6 +16741,10 @@
       <c r="C308" s="3" t="s">
         <v>894</v>
       </c>
+      <c r="D308" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in F major</v>
+      </c>
       <c r="E308" s="5" t="s">
         <v>872</v>
       </c>
@@ -16616,6 +16762,10 @@
       <c r="C309" s="3" t="s">
         <v>896</v>
       </c>
+      <c r="D309" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in F major</v>
+      </c>
       <c r="E309" s="5" t="s">
         <v>872</v>
       </c>
@@ -16636,6 +16786,10 @@
       <c r="C310" s="3" t="s">
         <v>898</v>
       </c>
+      <c r="D310" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in G major</v>
+      </c>
       <c r="E310" s="5" t="s">
         <v>872</v>
       </c>
@@ -16656,6 +16810,10 @@
       <c r="C311" s="3" t="s">
         <v>900</v>
       </c>
+      <c r="D311" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>March in G major</v>
+      </c>
       <c r="E311" s="5" t="s">
         <v>872</v>
       </c>
@@ -16701,6 +16859,10 @@
       <c r="C314" s="3" t="s">
         <v>905</v>
       </c>
+      <c r="D314" s="4" t="str">
+        <f t="shared" ref="D314:D316" si="4">E314&amp;" in "&amp;F314</f>
+        <v>Menuet in A major</v>
+      </c>
       <c r="E314" s="5" t="s">
         <v>906</v>
       </c>
@@ -16721,6 +16883,10 @@
       <c r="C315" s="3" t="s">
         <v>905</v>
       </c>
+      <c r="D315" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>Menuet in A major</v>
+      </c>
       <c r="E315" s="5" t="s">
         <v>906</v>
       </c>
@@ -16741,6 +16907,10 @@
       <c r="C316" s="3" t="s">
         <v>909</v>
       </c>
+      <c r="D316" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>Menuet in C major</v>
+      </c>
       <c r="E316" s="5" t="s">
         <v>906</v>
       </c>
@@ -16784,6 +16954,10 @@
       <c r="C318" s="3" t="s">
         <v>914</v>
       </c>
+      <c r="D318" s="4" t="str">
+        <f t="shared" ref="D318:D332" si="5">E318&amp;" in "&amp;F318</f>
+        <v>Menuet in C major</v>
+      </c>
       <c r="E318" s="5" t="s">
         <v>906</v>
       </c>
@@ -16804,6 +16978,10 @@
       <c r="C319" s="3" t="s">
         <v>916</v>
       </c>
+      <c r="D319" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in C major</v>
+      </c>
       <c r="E319" s="5" t="s">
         <v>906</v>
       </c>
@@ -16870,6 +17048,10 @@
       <c r="C322" s="3" t="s">
         <v>924</v>
       </c>
+      <c r="D322" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in C major</v>
+      </c>
       <c r="E322" s="5" t="s">
         <v>906</v>
       </c>
@@ -16887,6 +17069,10 @@
       <c r="C323" s="3" t="s">
         <v>926</v>
       </c>
+      <c r="D323" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in C major</v>
+      </c>
       <c r="E323" s="5" t="s">
         <v>906</v>
       </c>
@@ -16913,6 +17099,10 @@
       <c r="C324" s="3" t="s">
         <v>931</v>
       </c>
+      <c r="D324" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E324" s="5" t="s">
         <v>906</v>
       </c>
@@ -16933,6 +17123,10 @@
       <c r="C325" s="3" t="s">
         <v>931</v>
       </c>
+      <c r="D325" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E325" s="5" t="s">
         <v>906</v>
       </c>
@@ -16953,6 +17147,10 @@
       <c r="C326" s="3" t="s">
         <v>934</v>
       </c>
+      <c r="D326" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E326" s="5" t="s">
         <v>906</v>
       </c>
@@ -16973,6 +17171,10 @@
       <c r="C327" s="3" t="s">
         <v>934</v>
       </c>
+      <c r="D327" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E327" s="5" t="s">
         <v>906</v>
       </c>
@@ -16993,6 +17195,10 @@
       <c r="C328" s="3" t="s">
         <v>937</v>
       </c>
+      <c r="D328" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E328" s="5" t="s">
         <v>906</v>
       </c>
@@ -17013,6 +17219,10 @@
       <c r="C329" s="3" t="s">
         <v>940</v>
       </c>
+      <c r="D329" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E329" s="5" t="s">
         <v>906</v>
       </c>
@@ -17033,6 +17243,10 @@
       <c r="C330" s="3" t="s">
         <v>942</v>
       </c>
+      <c r="D330" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E330" s="5" t="s">
         <v>906</v>
       </c>
@@ -17053,6 +17267,10 @@
       <c r="C331" s="3" t="s">
         <v>944</v>
       </c>
+      <c r="D331" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E331" s="5" t="s">
         <v>906</v>
       </c>
@@ -17073,6 +17291,10 @@
       <c r="C332" s="3" t="s">
         <v>947</v>
       </c>
+      <c r="D332" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E332" s="5" t="s">
         <v>906</v>
       </c>
@@ -17113,6 +17335,10 @@
       <c r="C334" s="3" t="s">
         <v>953</v>
       </c>
+      <c r="D334" s="4" t="str">
+        <f t="shared" ref="D334:D341" si="6">E334&amp;" in "&amp;F334</f>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E334" s="5" t="s">
         <v>906</v>
       </c>
@@ -17133,6 +17359,10 @@
       <c r="C335" s="3" t="s">
         <v>955</v>
       </c>
+      <c r="D335" s="4" t="str">
+        <f t="shared" si="6"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E335" s="5" t="s">
         <v>906</v>
       </c>
@@ -17153,6 +17383,10 @@
       <c r="C336" s="3" t="s">
         <v>957</v>
       </c>
+      <c r="D336" s="4" t="str">
+        <f t="shared" si="6"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E336" s="5" t="s">
         <v>906</v>
       </c>
@@ -17170,6 +17404,10 @@
       <c r="C337" s="3" t="s">
         <v>959</v>
       </c>
+      <c r="D337" s="4" t="str">
+        <f t="shared" si="6"/>
+        <v>Menuet in D major</v>
+      </c>
       <c r="E337" s="5" t="s">
         <v>906</v>
       </c>
@@ -17196,6 +17434,10 @@
       <c r="C338" s="3" t="s">
         <v>964</v>
       </c>
+      <c r="D338" s="4" t="str">
+        <f t="shared" si="6"/>
+        <v>Menuet in E-flat major</v>
+      </c>
       <c r="E338" s="5" t="s">
         <v>906</v>
       </c>
@@ -17216,6 +17458,10 @@
       <c r="C339" s="3" t="s">
         <v>966</v>
       </c>
+      <c r="D339" s="4" t="str">
+        <f t="shared" si="6"/>
+        <v>Menuet in F major</v>
+      </c>
       <c r="E339" s="5" t="s">
         <v>906</v>
       </c>
@@ -17236,6 +17482,10 @@
       <c r="C340" s="3" t="s">
         <v>968</v>
       </c>
+      <c r="D340" s="4" t="str">
+        <f t="shared" si="6"/>
+        <v>Menuet in F major</v>
+      </c>
       <c r="E340" s="5" t="s">
         <v>906</v>
       </c>
@@ -17256,6 +17506,10 @@
       <c r="C341" s="3" t="s">
         <v>970</v>
       </c>
+      <c r="D341" s="4" t="str">
+        <f t="shared" si="6"/>
+        <v>Menuet in F major</v>
+      </c>
       <c r="E341" s="5" t="s">
         <v>906</v>
       </c>
@@ -17296,6 +17550,10 @@
       <c r="C343" s="3" t="s">
         <v>975</v>
       </c>
+      <c r="D343" s="4" t="str">
+        <f t="shared" ref="D343:D347" si="7">E343&amp;" in "&amp;F343</f>
+        <v>Menuet in F major</v>
+      </c>
       <c r="E343" s="5" t="s">
         <v>906</v>
       </c>
@@ -17316,6 +17574,10 @@
       <c r="C344" s="3" t="s">
         <v>977</v>
       </c>
+      <c r="D344" s="4" t="str">
+        <f t="shared" si="7"/>
+        <v>Menuet in G major</v>
+      </c>
       <c r="E344" s="5" t="s">
         <v>906</v>
       </c>
@@ -17336,6 +17598,10 @@
       <c r="C345" s="3" t="s">
         <v>979</v>
       </c>
+      <c r="D345" s="4" t="str">
+        <f t="shared" si="7"/>
+        <v>Menuet in G major</v>
+      </c>
       <c r="E345" s="5" t="s">
         <v>906</v>
       </c>
@@ -17362,6 +17628,10 @@
       <c r="C346" s="3" t="s">
         <v>984</v>
       </c>
+      <c r="D346" s="4" t="str">
+        <f t="shared" si="7"/>
+        <v>Menuet in G major</v>
+      </c>
       <c r="E346" s="5" t="s">
         <v>906</v>
       </c>
@@ -17382,6 +17652,10 @@
       <c r="C347" s="3" t="s">
         <v>986</v>
       </c>
+      <c r="D347" s="4" t="str">
+        <f t="shared" si="7"/>
+        <v>Menuet in G major</v>
+      </c>
       <c r="E347" s="5" t="s">
         <v>906</v>
       </c>
@@ -17448,6 +17722,10 @@
       <c r="C350" s="3" t="s">
         <v>994</v>
       </c>
+      <c r="D350" s="4" t="str">
+        <f t="shared" ref="D350:D352" si="8">E350&amp;" in "&amp;F350</f>
+        <v>Menuet in G major</v>
+      </c>
       <c r="E350" s="5" t="s">
         <v>906</v>
       </c>
@@ -17468,6 +17746,10 @@
       <c r="C351" s="3" t="s">
         <v>996</v>
       </c>
+      <c r="D351" s="4" t="str">
+        <f t="shared" si="8"/>
+        <v>Menuet in G major</v>
+      </c>
       <c r="E351" s="5" t="s">
         <v>906</v>
       </c>
@@ -17488,6 +17770,10 @@
       <c r="C352" s="3" t="s">
         <v>998</v>
       </c>
+      <c r="D352" s="4" t="str">
+        <f t="shared" si="8"/>
+        <v>Menuet in G major</v>
+      </c>
       <c r="E352" s="5" t="s">
         <v>906</v>
       </c>
@@ -17693,7 +17979,6 @@
       <c r="E363" s="5" t="s">
         <v>1029</v>
       </c>
-      <c r="F363" s="2"/>
       <c r="G363" s="6" t="s">
         <v>1030</v>
       </c>
@@ -19066,7 +19351,7 @@
         <v>1258</v>
       </c>
       <c r="D436" s="4" t="str">
-        <f t="shared" ref="D436:D475" si="0">E436&amp;" in "&amp;F436</f>
+        <f t="shared" ref="D436:D475" si="9">E436&amp;" in "&amp;F436</f>
         <v>Sonata in A major</v>
       </c>
       <c r="E436" s="5" t="s">
@@ -19093,7 +19378,7 @@
         <v>1260</v>
       </c>
       <c r="D437" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E437" s="5" t="s">
@@ -19117,7 +19402,7 @@
         <v>1262</v>
       </c>
       <c r="D438" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E438" s="5" t="s">
@@ -19141,7 +19426,7 @@
         <v>1264</v>
       </c>
       <c r="D439" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E439" s="5" t="s">
@@ -19165,7 +19450,7 @@
         <v>1266</v>
       </c>
       <c r="D440" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E440" s="5" t="s">
@@ -19189,7 +19474,7 @@
         <v>1268</v>
       </c>
       <c r="D441" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E441" s="5" t="s">
@@ -19213,7 +19498,7 @@
         <v>1270</v>
       </c>
       <c r="D442" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E442" s="5" t="s">
@@ -19237,7 +19522,7 @@
         <v>1272</v>
       </c>
       <c r="D443" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E443" s="5" t="s">
@@ -19261,7 +19546,7 @@
         <v>1274</v>
       </c>
       <c r="D444" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E444" s="5" t="s">
@@ -19285,7 +19570,7 @@
         <v>1276</v>
       </c>
       <c r="D445" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E445" s="5" t="s">
@@ -19309,7 +19594,7 @@
         <v>1279</v>
       </c>
       <c r="D446" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E446" s="5" t="s">
@@ -19333,7 +19618,7 @@
         <v>1282</v>
       </c>
       <c r="D447" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A major</v>
       </c>
       <c r="E447" s="5" t="s">
@@ -19357,7 +19642,7 @@
         <v>1284</v>
       </c>
       <c r="D448" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E448" s="5" t="s">
@@ -19384,7 +19669,7 @@
         <v>1286</v>
       </c>
       <c r="D449" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E449" s="5" t="s">
@@ -19411,7 +19696,7 @@
         <v>1288</v>
       </c>
       <c r="D450" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E450" s="5" t="s">
@@ -19435,7 +19720,7 @@
         <v>1290</v>
       </c>
       <c r="D451" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E451" s="5" t="s">
@@ -19459,7 +19744,7 @@
         <v>1292</v>
       </c>
       <c r="D452" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E452" s="5" t="s">
@@ -19486,7 +19771,7 @@
         <v>1296</v>
       </c>
       <c r="D453" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E453" s="5" t="s">
@@ -19510,7 +19795,7 @@
         <v>1298</v>
       </c>
       <c r="D454" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E454" s="5" t="s">
@@ -19534,7 +19819,7 @@
         <v>1300</v>
       </c>
       <c r="D455" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E455" s="5" t="s">
@@ -19558,7 +19843,7 @@
         <v>1302</v>
       </c>
       <c r="D456" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E456" s="5" t="s">
@@ -19582,7 +19867,7 @@
         <v>1304</v>
       </c>
       <c r="D457" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E457" s="5" t="s">
@@ -19606,7 +19891,7 @@
         <v>1306</v>
       </c>
       <c r="D458" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E458" s="5" t="s">
@@ -19630,7 +19915,7 @@
         <v>1308</v>
       </c>
       <c r="D459" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E459" s="5" t="s">
@@ -19654,7 +19939,7 @@
         <v>1311</v>
       </c>
       <c r="D460" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A minor</v>
       </c>
       <c r="E460" s="5" t="s">
@@ -19678,7 +19963,7 @@
         <v>1314</v>
       </c>
       <c r="D461" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in A-flat major</v>
       </c>
       <c r="E461" s="5" t="s">
@@ -19702,7 +19987,7 @@
         <v>1317</v>
       </c>
       <c r="D462" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E462" s="5" t="s">
@@ -19729,7 +20014,7 @@
         <v>1319</v>
       </c>
       <c r="D463" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E463" s="5" t="s">
@@ -19753,7 +20038,7 @@
         <v>1321</v>
       </c>
       <c r="D464" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E464" s="5" t="s">
@@ -19777,7 +20062,7 @@
         <v>1323</v>
       </c>
       <c r="D465" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E465" s="5" t="s">
@@ -19801,7 +20086,7 @@
         <v>1325</v>
       </c>
       <c r="D466" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E466" s="5" t="s">
@@ -19825,7 +20110,7 @@
         <v>1327</v>
       </c>
       <c r="D467" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E467" s="5" t="s">
@@ -19846,7 +20131,7 @@
         <v>1328</v>
       </c>
       <c r="D468" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E468" s="5" t="s">
@@ -19876,7 +20161,7 @@
         <v>1331</v>
       </c>
       <c r="D469" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E469" s="5" t="s">
@@ -19900,7 +20185,7 @@
         <v>1333</v>
       </c>
       <c r="D470" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B minor</v>
       </c>
       <c r="E470" s="5" t="s">
@@ -19924,7 +20209,7 @@
         <v>1335</v>
       </c>
       <c r="D471" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E471" s="5" t="s">
@@ -19951,7 +20236,7 @@
         <v>1337</v>
       </c>
       <c r="D472" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E472" s="5" t="s">
@@ -19978,7 +20263,7 @@
         <v>1339</v>
       </c>
       <c r="D473" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E473" s="5" t="s">
@@ -20002,7 +20287,7 @@
         <v>1341</v>
       </c>
       <c r="D474" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E474" s="5" t="s">
@@ -20026,7 +20311,7 @@
         <v>1343</v>
       </c>
       <c r="D475" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E475" s="5" t="s">
@@ -20097,7 +20382,7 @@
         <v>1350</v>
       </c>
       <c r="D478" s="4" t="str">
-        <f t="shared" ref="D478:D509" si="1">E478&amp;" in "&amp;F478</f>
+        <f t="shared" ref="D478:D509" si="10">E478&amp;" in "&amp;F478</f>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E478" s="5" t="s">
@@ -20121,7 +20406,7 @@
         <v>1352</v>
       </c>
       <c r="D479" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E479" s="5" t="s">
@@ -20145,7 +20430,7 @@
         <v>1355</v>
       </c>
       <c r="D480" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E480" s="5" t="s">
@@ -20169,7 +20454,7 @@
         <v>1357</v>
       </c>
       <c r="D481" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E481" s="5" t="s">
@@ -20193,7 +20478,7 @@
         <v>1359</v>
       </c>
       <c r="D482" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E482" s="5" t="s">
@@ -20217,7 +20502,7 @@
         <v>1361</v>
       </c>
       <c r="D483" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E483" s="5" t="s">
@@ -20241,7 +20526,7 @@
         <v>1363</v>
       </c>
       <c r="D484" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E484" s="5" t="s">
@@ -20265,7 +20550,7 @@
         <v>1365</v>
       </c>
       <c r="D485" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E485" s="5" t="s">
@@ -20289,7 +20574,7 @@
         <v>1367</v>
       </c>
       <c r="D486" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E486" s="5" t="s">
@@ -20313,7 +20598,7 @@
         <v>1369</v>
       </c>
       <c r="D487" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E487" s="5" t="s">
@@ -20337,7 +20622,7 @@
         <v>1371</v>
       </c>
       <c r="D488" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E488" s="5" t="s">
@@ -20361,7 +20646,7 @@
         <v>1373</v>
       </c>
       <c r="D489" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E489" s="5" t="s">
@@ -20385,7 +20670,7 @@
         <v>1375</v>
       </c>
       <c r="D490" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E490" s="5" t="s">
@@ -20409,7 +20694,7 @@
         <v>1378</v>
       </c>
       <c r="D491" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E491" s="5" t="s">
@@ -20433,7 +20718,7 @@
         <v>1380</v>
       </c>
       <c r="D492" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E492" s="5" t="s">
@@ -20457,7 +20742,7 @@
         <v>1382</v>
       </c>
       <c r="D493" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in B-flat major</v>
       </c>
       <c r="E493" s="5" t="s">
@@ -20478,7 +20763,7 @@
         <v>1383</v>
       </c>
       <c r="D494" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E494" s="5" t="s">
@@ -20508,7 +20793,7 @@
         <v>1387</v>
       </c>
       <c r="D495" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E495" s="5" t="s">
@@ -20535,7 +20820,7 @@
         <v>1389</v>
       </c>
       <c r="D496" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E496" s="5" t="s">
@@ -20562,7 +20847,7 @@
         <v>1391</v>
       </c>
       <c r="D497" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E497" s="5" t="s">
@@ -20586,7 +20871,7 @@
         <v>1393</v>
       </c>
       <c r="D498" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E498" s="5" t="s">
@@ -20610,7 +20895,7 @@
         <v>1395</v>
       </c>
       <c r="D499" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E499" s="5" t="s">
@@ -20634,7 +20919,7 @@
         <v>1397</v>
       </c>
       <c r="D500" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E500" s="5" t="s">
@@ -20658,7 +20943,7 @@
         <v>1399</v>
       </c>
       <c r="D501" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E501" s="5" t="s">
@@ -20682,7 +20967,7 @@
         <v>1401</v>
       </c>
       <c r="D502" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E502" s="5" t="s">
@@ -20706,7 +20991,7 @@
         <v>1403</v>
       </c>
       <c r="D503" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E503" s="5" t="s">
@@ -20730,7 +21015,7 @@
         <v>1405</v>
       </c>
       <c r="D504" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E504" s="5" t="s">
@@ -20754,7 +21039,7 @@
         <v>1407</v>
       </c>
       <c r="D505" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E505" s="5" t="s">
@@ -20778,7 +21063,7 @@
         <v>1409</v>
       </c>
       <c r="D506" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E506" s="5" t="s">
@@ -20802,7 +21087,7 @@
         <v>1411</v>
       </c>
       <c r="D507" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E507" s="5" t="s">
@@ -20826,7 +21111,7 @@
         <v>1413</v>
       </c>
       <c r="D508" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E508" s="5" t="s">
@@ -20850,7 +21135,7 @@
         <v>1415</v>
       </c>
       <c r="D509" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E509" s="5" t="s">
@@ -20874,7 +21159,7 @@
         <v>1417</v>
       </c>
       <c r="D510" s="4" t="str">
-        <f t="shared" ref="D510:D534" si="2">E510&amp;" in "&amp;F510</f>
+        <f t="shared" ref="D510:D534" si="11">E510&amp;" in "&amp;F510</f>
         <v>Sonata in C major</v>
       </c>
       <c r="E510" s="5" t="s">
@@ -20898,7 +21183,7 @@
         <v>1419</v>
       </c>
       <c r="D511" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E511" s="5" t="s">
@@ -20922,7 +21207,7 @@
         <v>1421</v>
       </c>
       <c r="D512" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E512" s="5" t="s">
@@ -20946,7 +21231,7 @@
         <v>1423</v>
       </c>
       <c r="D513" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E513" s="5" t="s">
@@ -20970,7 +21255,7 @@
         <v>1426</v>
       </c>
       <c r="D514" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E514" s="5" t="s">
@@ -20994,7 +21279,7 @@
         <v>1428</v>
       </c>
       <c r="D515" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E515" s="5" t="s">
@@ -21018,7 +21303,7 @@
         <v>1430</v>
       </c>
       <c r="D516" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E516" s="5" t="s">
@@ -21042,7 +21327,7 @@
         <v>1432</v>
       </c>
       <c r="D517" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E517" s="5" t="s">
@@ -21066,7 +21351,7 @@
         <v>1434</v>
       </c>
       <c r="D518" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E518" s="5" t="s">
@@ -21090,7 +21375,7 @@
         <v>1436</v>
       </c>
       <c r="D519" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C major</v>
       </c>
       <c r="E519" s="5" t="s">
@@ -21114,7 +21399,7 @@
         <v>1438</v>
       </c>
       <c r="D520" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C minor</v>
       </c>
       <c r="E520" s="5" t="s">
@@ -21138,7 +21423,7 @@
         <v>1440</v>
       </c>
       <c r="D521" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C minor</v>
       </c>
       <c r="E521" s="5" t="s">
@@ -21162,7 +21447,7 @@
         <v>1442</v>
       </c>
       <c r="D522" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C minor</v>
       </c>
       <c r="E522" s="5" t="s">
@@ -21186,7 +21471,7 @@
         <v>1444</v>
       </c>
       <c r="D523" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C minor</v>
       </c>
       <c r="E523" s="5" t="s">
@@ -21210,7 +21495,7 @@
         <v>1446</v>
       </c>
       <c r="D524" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C minor</v>
       </c>
       <c r="E524" s="5" t="s">
@@ -21234,7 +21519,7 @@
         <v>1448</v>
       </c>
       <c r="D525" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C minor</v>
       </c>
       <c r="E525" s="5" t="s">
@@ -21258,7 +21543,7 @@
         <v>1450</v>
       </c>
       <c r="D526" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in C minor</v>
       </c>
       <c r="E526" s="5" t="s">
@@ -21282,7 +21567,7 @@
         <v>1452</v>
       </c>
       <c r="D527" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E527" s="5" t="s">
@@ -21309,7 +21594,7 @@
         <v>1455</v>
       </c>
       <c r="D528" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E528" s="5" t="s">
@@ -21333,7 +21618,7 @@
         <v>1457</v>
       </c>
       <c r="D529" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E529" s="5" t="s">
@@ -21357,7 +21642,7 @@
         <v>1459</v>
       </c>
       <c r="D530" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E530" s="5" t="s">
@@ -21381,7 +21666,7 @@
         <v>1461</v>
       </c>
       <c r="D531" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E531" s="5" t="s">
@@ -21405,7 +21690,7 @@
         <v>1463</v>
       </c>
       <c r="D532" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E532" s="5" t="s">
@@ -21429,7 +21714,7 @@
         <v>1465</v>
       </c>
       <c r="D533" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E533" s="5" t="s">
@@ -21453,7 +21738,7 @@
         <v>1467</v>
       </c>
       <c r="D534" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E534" s="5" t="s">
@@ -21524,7 +21809,7 @@
         <v>1474</v>
       </c>
       <c r="D537" s="4" t="str">
-        <f t="shared" ref="D537:D568" si="3">E537&amp;" in "&amp;F537</f>
+        <f t="shared" ref="D537:D568" si="12">E537&amp;" in "&amp;F537</f>
         <v>Sonata in D major</v>
       </c>
       <c r="E537" s="5" t="s">
@@ -21548,7 +21833,7 @@
         <v>1476</v>
       </c>
       <c r="D538" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E538" s="5" t="s">
@@ -21572,7 +21857,7 @@
         <v>1478</v>
       </c>
       <c r="D539" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E539" s="5" t="s">
@@ -21596,7 +21881,7 @@
         <v>1480</v>
       </c>
       <c r="D540" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E540" s="5" t="s">
@@ -21620,7 +21905,7 @@
         <v>1482</v>
       </c>
       <c r="D541" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E541" s="5" t="s">
@@ -21644,7 +21929,7 @@
         <v>1484</v>
       </c>
       <c r="D542" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E542" s="5" t="s">
@@ -21668,7 +21953,7 @@
         <v>1486</v>
       </c>
       <c r="D543" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D major</v>
       </c>
       <c r="E543" s="5" t="s">
@@ -21692,7 +21977,7 @@
         <v>1488</v>
       </c>
       <c r="D544" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E544" s="5" t="s">
@@ -21719,7 +22004,7 @@
         <v>1490</v>
       </c>
       <c r="D545" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E545" s="5" t="s">
@@ -21749,7 +22034,7 @@
         <v>1493</v>
       </c>
       <c r="D546" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E546" s="5" t="s">
@@ -21776,7 +22061,7 @@
         <v>1495</v>
       </c>
       <c r="D547" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E547" s="5" t="s">
@@ -21800,7 +22085,7 @@
         <v>1497</v>
       </c>
       <c r="D548" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E548" s="5" t="s">
@@ -21824,7 +22109,7 @@
         <v>1499</v>
       </c>
       <c r="D549" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E549" s="5" t="s">
@@ -21848,7 +22133,7 @@
         <v>1501</v>
       </c>
       <c r="D550" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E550" s="5" t="s">
@@ -21872,7 +22157,7 @@
         <v>1503</v>
       </c>
       <c r="D551" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E551" s="5" t="s">
@@ -21896,7 +22181,7 @@
         <v>1505</v>
       </c>
       <c r="D552" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E552" s="5" t="s">
@@ -21920,7 +22205,7 @@
         <v>1507</v>
       </c>
       <c r="D553" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E553" s="5" t="s">
@@ -21944,7 +22229,7 @@
         <v>1509</v>
       </c>
       <c r="D554" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E554" s="5" t="s">
@@ -21968,7 +22253,7 @@
         <v>1511</v>
       </c>
       <c r="D555" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E555" s="5" t="s">
@@ -21992,7 +22277,7 @@
         <v>1513</v>
       </c>
       <c r="D556" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E556" s="5" t="s">
@@ -22016,7 +22301,7 @@
         <v>1515</v>
       </c>
       <c r="D557" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E557" s="5" t="s">
@@ -22040,7 +22325,7 @@
         <v>1517</v>
       </c>
       <c r="D558" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in D minor</v>
       </c>
       <c r="E558" s="5" t="s">
@@ -22064,7 +22349,7 @@
         <v>1519</v>
       </c>
       <c r="D559" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E major</v>
       </c>
       <c r="E559" s="5" t="s">
@@ -22088,7 +22373,7 @@
         <v>1521</v>
       </c>
       <c r="D560" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E major</v>
       </c>
       <c r="E560" s="5" t="s">
@@ -22112,7 +22397,7 @@
         <v>1523</v>
       </c>
       <c r="D561" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E major</v>
       </c>
       <c r="E561" s="5" t="s">
@@ -22136,7 +22421,7 @@
         <v>1525</v>
       </c>
       <c r="D562" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E major</v>
       </c>
       <c r="E562" s="5" t="s">
@@ -22160,7 +22445,7 @@
         <v>1528</v>
       </c>
       <c r="D563" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E major</v>
       </c>
       <c r="E563" s="5" t="s">
@@ -22184,7 +22469,7 @@
         <v>1530</v>
       </c>
       <c r="D564" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E major</v>
       </c>
       <c r="E564" s="5" t="s">
@@ -22208,7 +22493,7 @@
         <v>1532</v>
       </c>
       <c r="D565" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E major</v>
       </c>
       <c r="E565" s="5" t="s">
@@ -22232,7 +22517,7 @@
         <v>1534</v>
       </c>
       <c r="D566" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E major</v>
       </c>
       <c r="E566" s="5" t="s">
@@ -22256,7 +22541,7 @@
         <v>1536</v>
       </c>
       <c r="D567" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E567" s="5" t="s">
@@ -22283,7 +22568,7 @@
         <v>1538</v>
       </c>
       <c r="D568" s="4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E568" s="5" t="s">
@@ -22310,7 +22595,7 @@
         <v>1540</v>
       </c>
       <c r="D569" s="4" t="str">
-        <f t="shared" ref="D569:D600" si="4">E569&amp;" in "&amp;F569</f>
+        <f t="shared" ref="D569:D600" si="13">E569&amp;" in "&amp;F569</f>
         <v>Sonata in E minor</v>
       </c>
       <c r="E569" s="5" t="s">
@@ -22337,7 +22622,7 @@
         <v>1542</v>
       </c>
       <c r="D570" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E570" s="5" t="s">
@@ -22361,7 +22646,7 @@
         <v>1544</v>
       </c>
       <c r="D571" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E571" s="5" t="s">
@@ -22385,7 +22670,7 @@
         <v>1546</v>
       </c>
       <c r="D572" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E572" s="5" t="s">
@@ -22409,7 +22694,7 @@
         <v>1548</v>
       </c>
       <c r="D573" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E573" s="5" t="s">
@@ -22433,7 +22718,7 @@
         <v>1550</v>
       </c>
       <c r="D574" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E574" s="5" t="s">
@@ -22457,7 +22742,7 @@
         <v>1552</v>
       </c>
       <c r="D575" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E575" s="5" t="s">
@@ -22481,7 +22766,7 @@
         <v>1554</v>
       </c>
       <c r="D576" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E576" s="5" t="s">
@@ -22505,7 +22790,7 @@
         <v>1556</v>
       </c>
       <c r="D577" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E577" s="5" t="s">
@@ -22529,7 +22814,7 @@
         <v>1558</v>
       </c>
       <c r="D578" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E578" s="5" t="s">
@@ -22553,7 +22838,7 @@
         <v>1560</v>
       </c>
       <c r="D579" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E579" s="5" t="s">
@@ -22577,7 +22862,7 @@
         <v>1562</v>
       </c>
       <c r="D580" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E minor</v>
       </c>
       <c r="E580" s="5" t="s">
@@ -22601,7 +22886,7 @@
         <v>1564</v>
       </c>
       <c r="D581" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E581" s="5" t="s">
@@ -22628,7 +22913,7 @@
         <v>1566</v>
       </c>
       <c r="D582" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E582" s="5" t="s">
@@ -22652,7 +22937,7 @@
         <v>1568</v>
       </c>
       <c r="D583" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E583" s="5" t="s">
@@ -22676,7 +22961,7 @@
         <v>1570</v>
       </c>
       <c r="D584" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E584" s="5" t="s">
@@ -22700,7 +22985,7 @@
         <v>1572</v>
       </c>
       <c r="D585" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E585" s="5" t="s">
@@ -22724,7 +23009,7 @@
         <v>1574</v>
       </c>
       <c r="D586" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E586" s="5" t="s">
@@ -22748,7 +23033,7 @@
         <v>1576</v>
       </c>
       <c r="D587" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E587" s="5" t="s">
@@ -22772,7 +23057,7 @@
         <v>1578</v>
       </c>
       <c r="D588" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E588" s="5" t="s">
@@ -22796,7 +23081,7 @@
         <v>1580</v>
       </c>
       <c r="D589" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E589" s="5" t="s">
@@ -22820,7 +23105,7 @@
         <v>1582</v>
       </c>
       <c r="D590" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E590" s="5" t="s">
@@ -22844,7 +23129,7 @@
         <v>1584</v>
       </c>
       <c r="D591" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E591" s="5" t="s">
@@ -22868,7 +23153,7 @@
         <v>1586</v>
       </c>
       <c r="D592" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E592" s="5" t="s">
@@ -22892,7 +23177,7 @@
         <v>1588</v>
       </c>
       <c r="D593" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in E-flat major</v>
       </c>
       <c r="E593" s="5" t="s">
@@ -22916,7 +23201,7 @@
         <v>1590</v>
       </c>
       <c r="D594" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E594" s="5" t="s">
@@ -22943,7 +23228,7 @@
         <v>1592</v>
       </c>
       <c r="D595" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E595" s="5" t="s">
@@ -22967,7 +23252,7 @@
         <v>1594</v>
       </c>
       <c r="D596" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E596" s="5" t="s">
@@ -22991,7 +23276,7 @@
         <v>1596</v>
       </c>
       <c r="D597" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E597" s="5" t="s">
@@ -23015,7 +23300,7 @@
         <v>1598</v>
       </c>
       <c r="D598" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E598" s="5" t="s">
@@ -23039,7 +23324,7 @@
         <v>1600</v>
       </c>
       <c r="D599" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E599" s="5" t="s">
@@ -23063,7 +23348,7 @@
         <v>1602</v>
       </c>
       <c r="D600" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E600" s="5" t="s">
@@ -23087,7 +23372,7 @@
         <v>1604</v>
       </c>
       <c r="D601" s="4" t="str">
-        <f t="shared" ref="D601:D631" si="5">E601&amp;" in "&amp;F601</f>
+        <f t="shared" ref="D601:D631" si="14">E601&amp;" in "&amp;F601</f>
         <v>Sonata in F major</v>
       </c>
       <c r="E601" s="5" t="s">
@@ -23111,7 +23396,7 @@
         <v>1606</v>
       </c>
       <c r="D602" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E602" s="5" t="s">
@@ -23135,7 +23420,7 @@
         <v>1609</v>
       </c>
       <c r="D603" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E603" s="5" t="s">
@@ -23159,7 +23444,7 @@
         <v>1611</v>
       </c>
       <c r="D604" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E604" s="5" t="s">
@@ -23183,7 +23468,7 @@
         <v>1613</v>
       </c>
       <c r="D605" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E605" s="5" t="s">
@@ -23207,7 +23492,7 @@
         <v>1615</v>
       </c>
       <c r="D606" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E606" s="5" t="s">
@@ -23231,7 +23516,7 @@
         <v>1617</v>
       </c>
       <c r="D607" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E607" s="5" t="s">
@@ -23255,7 +23540,7 @@
         <v>1619</v>
       </c>
       <c r="D608" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E608" s="5" t="s">
@@ -23279,7 +23564,7 @@
         <v>1621</v>
       </c>
       <c r="D609" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E609" s="5" t="s">
@@ -23303,7 +23588,7 @@
         <v>1623</v>
       </c>
       <c r="D610" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E610" s="5" t="s">
@@ -23327,7 +23612,7 @@
         <v>1625</v>
       </c>
       <c r="D611" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E611" s="5" t="s">
@@ -23351,7 +23636,7 @@
         <v>1627</v>
       </c>
       <c r="D612" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E612" s="5" t="s">
@@ -23375,7 +23660,7 @@
         <v>1629</v>
       </c>
       <c r="D613" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E613" s="5" t="s">
@@ -23399,7 +23684,7 @@
         <v>1630</v>
       </c>
       <c r="D614" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E614" s="5" t="s">
@@ -23423,7 +23708,7 @@
         <v>1632</v>
       </c>
       <c r="D615" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F major</v>
       </c>
       <c r="E615" s="5" t="s">
@@ -23447,7 +23732,7 @@
         <v>1634</v>
       </c>
       <c r="D616" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F minor</v>
       </c>
       <c r="E616" s="5" t="s">
@@ -23471,7 +23756,7 @@
         <v>1636</v>
       </c>
       <c r="D617" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F minor</v>
       </c>
       <c r="E617" s="5" t="s">
@@ -23495,7 +23780,7 @@
         <v>1638</v>
       </c>
       <c r="D618" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F minor</v>
       </c>
       <c r="E618" s="5" t="s">
@@ -23519,7 +23804,7 @@
         <v>1640</v>
       </c>
       <c r="D619" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in F-sharp minor</v>
       </c>
       <c r="E619" s="5" t="s">
@@ -23543,7 +23828,7 @@
         <v>1642</v>
       </c>
       <c r="D620" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E620" s="5" t="s">
@@ -23567,7 +23852,7 @@
         <v>1644</v>
       </c>
       <c r="D621" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E621" s="5" t="s">
@@ -23591,7 +23876,7 @@
         <v>1646</v>
       </c>
       <c r="D622" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E622" s="5" t="s">
@@ -23618,7 +23903,7 @@
         <v>1648</v>
       </c>
       <c r="D623" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E623" s="5" t="s">
@@ -23642,7 +23927,7 @@
         <v>1650</v>
       </c>
       <c r="D624" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E624" s="5" t="s">
@@ -23666,7 +23951,7 @@
         <v>1652</v>
       </c>
       <c r="D625" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E625" s="5" t="s">
@@ -23690,7 +23975,7 @@
         <v>1654</v>
       </c>
       <c r="D626" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E626" s="5" t="s">
@@ -23714,7 +23999,7 @@
         <v>1656</v>
       </c>
       <c r="D627" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E627" s="5" t="s">
@@ -23738,7 +24023,7 @@
         <v>1658</v>
       </c>
       <c r="D628" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E628" s="5" t="s">
@@ -23762,7 +24047,7 @@
         <v>1660</v>
       </c>
       <c r="D629" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E629" s="5" t="s">
@@ -23786,7 +24071,7 @@
         <v>1662</v>
       </c>
       <c r="D630" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E630" s="5" t="s">
@@ -23810,7 +24095,7 @@
         <v>1664</v>
       </c>
       <c r="D631" s="4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E631" s="5" t="s">
@@ -23881,7 +24166,7 @@
         <v>1671</v>
       </c>
       <c r="D634" s="4" t="str">
-        <f t="shared" ref="D634:D659" si="6">E634&amp;" in "&amp;F634</f>
+        <f t="shared" ref="D634:D659" si="15">E634&amp;" in "&amp;F634</f>
         <v>Sonata in G major</v>
       </c>
       <c r="E634" s="5" t="s">
@@ -23905,7 +24190,7 @@
         <v>1673</v>
       </c>
       <c r="D635" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E635" s="5" t="s">
@@ -23929,7 +24214,7 @@
         <v>1675</v>
       </c>
       <c r="D636" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E636" s="5" t="s">
@@ -23953,7 +24238,7 @@
         <v>1677</v>
       </c>
       <c r="D637" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E637" s="5" t="s">
@@ -23977,7 +24262,7 @@
         <v>1679</v>
       </c>
       <c r="D638" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E638" s="5" t="s">
@@ -23998,7 +24283,7 @@
         <v>1680</v>
       </c>
       <c r="D639" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E639" s="5" t="s">
@@ -24028,7 +24313,7 @@
         <v>1683</v>
       </c>
       <c r="D640" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E640" s="5" t="s">
@@ -24052,7 +24337,7 @@
         <v>1685</v>
       </c>
       <c r="D641" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E641" s="5" t="s">
@@ -24076,7 +24361,7 @@
         <v>1687</v>
       </c>
       <c r="D642" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E642" s="5" t="s">
@@ -24100,7 +24385,7 @@
         <v>1689</v>
       </c>
       <c r="D643" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E643" s="5" t="s">
@@ -24124,7 +24409,7 @@
         <v>1690</v>
       </c>
       <c r="D644" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E644" s="5" t="s">
@@ -24148,7 +24433,7 @@
         <v>1692</v>
       </c>
       <c r="D645" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E645" s="5" t="s">
@@ -24172,7 +24457,7 @@
         <v>1694</v>
       </c>
       <c r="D646" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E646" s="5" t="s">
@@ -24196,7 +24481,7 @@
         <v>1696</v>
       </c>
       <c r="D647" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E647" s="5" t="s">
@@ -24220,7 +24505,7 @@
         <v>1698</v>
       </c>
       <c r="D648" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E648" s="5" t="s">
@@ -24244,7 +24529,7 @@
         <v>1700</v>
       </c>
       <c r="D649" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G major</v>
       </c>
       <c r="E649" s="5" t="s">
@@ -24268,7 +24553,7 @@
         <v>1702</v>
       </c>
       <c r="D650" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E650" s="5" t="s">
@@ -24292,7 +24577,7 @@
         <v>1704</v>
       </c>
       <c r="D651" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E651" s="5" t="s">
@@ -24316,7 +24601,7 @@
         <v>1706</v>
       </c>
       <c r="D652" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E652" s="5" t="s">
@@ -24340,7 +24625,7 @@
         <v>1708</v>
       </c>
       <c r="D653" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E653" s="5" t="s">
@@ -24364,7 +24649,7 @@
         <v>1710</v>
       </c>
       <c r="D654" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E654" s="5" t="s">
@@ -24388,7 +24673,7 @@
         <v>1712</v>
       </c>
       <c r="D655" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E655" s="5" t="s">
@@ -24412,7 +24697,7 @@
         <v>1714</v>
       </c>
       <c r="D656" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E656" s="5" t="s">
@@ -24436,7 +24721,7 @@
         <v>1717</v>
       </c>
       <c r="D657" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E657" s="5" t="s">
@@ -24460,7 +24745,7 @@
         <v>1719</v>
       </c>
       <c r="D658" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E658" s="5" t="s">
@@ -24484,7 +24769,7 @@
         <v>1721</v>
       </c>
       <c r="D659" s="4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>Sonata in G minor</v>
       </c>
       <c r="E659" s="5" t="s">
@@ -24934,7 +25219,7 @@
         <v>1771</v>
       </c>
       <c r="D685" s="4" t="str">
-        <f t="shared" ref="D685:D710" si="7">E685&amp;" in "&amp;F685</f>
+        <f t="shared" ref="D685:D710" si="16">E685&amp;" in "&amp;F685</f>
         <v>Sonatina in B-flat major</v>
       </c>
       <c r="E685" s="5" t="s">
@@ -24958,7 +25243,7 @@
         <v>1774</v>
       </c>
       <c r="D686" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in B-flat major</v>
       </c>
       <c r="E686" s="5" t="s">
@@ -24982,7 +25267,7 @@
         <v>1776</v>
       </c>
       <c r="D687" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in C major</v>
       </c>
       <c r="E687" s="5" t="s">
@@ -25006,7 +25291,7 @@
         <v>1778</v>
       </c>
       <c r="D688" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in C major</v>
       </c>
       <c r="E688" s="5" t="s">
@@ -25030,7 +25315,7 @@
         <v>1781</v>
       </c>
       <c r="D689" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in C major</v>
       </c>
       <c r="E689" s="5" t="s">
@@ -25054,7 +25339,7 @@
         <v>1783</v>
       </c>
       <c r="D690" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in D major</v>
       </c>
       <c r="E690" s="5" t="s">
@@ -25081,7 +25366,7 @@
         <v>1785</v>
       </c>
       <c r="D691" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in D major</v>
       </c>
       <c r="E691" s="5" t="s">
@@ -25105,7 +25390,7 @@
         <v>1787</v>
       </c>
       <c r="D692" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in D major</v>
       </c>
       <c r="E692" s="5" t="s">
@@ -25129,7 +25414,7 @@
         <v>1789</v>
       </c>
       <c r="D693" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in D major</v>
       </c>
       <c r="E693" s="5" t="s">
@@ -25153,7 +25438,7 @@
         <v>1791</v>
       </c>
       <c r="D694" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in D major</v>
       </c>
       <c r="E694" s="5" t="s">
@@ -25177,7 +25462,7 @@
         <v>1793</v>
       </c>
       <c r="D695" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in D minor</v>
       </c>
       <c r="E695" s="5" t="s">
@@ -25201,7 +25486,7 @@
         <v>1796</v>
       </c>
       <c r="D696" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in D minor</v>
       </c>
       <c r="E696" s="5" t="s">
@@ -25225,7 +25510,7 @@
         <v>1798</v>
       </c>
       <c r="D697" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in E major</v>
       </c>
       <c r="E697" s="5" t="s">
@@ -25249,7 +25534,7 @@
         <v>1800</v>
       </c>
       <c r="D698" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in E major</v>
       </c>
       <c r="E698" s="5" t="s">
@@ -25273,7 +25558,7 @@
         <v>1802</v>
       </c>
       <c r="D699" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in E minor</v>
       </c>
       <c r="E699" s="5" t="s">
@@ -25300,7 +25585,7 @@
         <v>1804</v>
       </c>
       <c r="D700" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in E-flat major</v>
       </c>
       <c r="E700" s="5" t="s">
@@ -25327,7 +25612,7 @@
         <v>1806</v>
       </c>
       <c r="D701" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in E-flat major</v>
       </c>
       <c r="E701" s="5" t="s">
@@ -25351,7 +25636,7 @@
         <v>1808</v>
       </c>
       <c r="D702" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in E-flat major</v>
       </c>
       <c r="E702" s="5" t="s">
@@ -25375,7 +25660,7 @@
         <v>1810</v>
       </c>
       <c r="D703" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in F major</v>
       </c>
       <c r="E703" s="5" t="s">
@@ -25402,7 +25687,7 @@
         <v>1812</v>
       </c>
       <c r="D704" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in F major</v>
       </c>
       <c r="E704" s="5" t="s">
@@ -25426,7 +25711,7 @@
         <v>1814</v>
       </c>
       <c r="D705" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in F major</v>
       </c>
       <c r="E705" s="5" t="s">
@@ -25450,7 +25735,7 @@
         <v>1816</v>
       </c>
       <c r="D706" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in F major</v>
       </c>
       <c r="E706" s="5" t="s">
@@ -25474,7 +25759,7 @@
         <v>1818</v>
       </c>
       <c r="D707" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in G major</v>
       </c>
       <c r="E707" s="5" t="s">
@@ -25501,7 +25786,7 @@
         <v>1820</v>
       </c>
       <c r="D708" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in G major</v>
       </c>
       <c r="E708" s="5" t="s">
@@ -25525,7 +25810,7 @@
         <v>1822</v>
       </c>
       <c r="D709" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in G major</v>
       </c>
       <c r="E709" s="5" t="s">
@@ -25549,7 +25834,7 @@
         <v>1824</v>
       </c>
       <c r="D710" s="4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>Sonatina in G major</v>
       </c>
       <c r="E710" s="5" t="s">
@@ -25614,7 +25899,7 @@
         <v>1831</v>
       </c>
       <c r="D713" s="4" t="str">
-        <f t="shared" ref="D713:D725" si="8">E713&amp;" in "&amp;F713</f>
+        <f t="shared" ref="D713:D725" si="17">E713&amp;" in "&amp;F713</f>
         <v>Symphony in D major</v>
       </c>
       <c r="E713" s="5" t="s">
@@ -25638,7 +25923,7 @@
         <v>1833</v>
       </c>
       <c r="D714" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in E minor</v>
       </c>
       <c r="E714" s="5" t="s">
@@ -25662,7 +25947,7 @@
         <v>1835</v>
       </c>
       <c r="D715" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in E minor</v>
       </c>
       <c r="E715" s="5" t="s">
@@ -25686,7 +25971,7 @@
         <v>1837</v>
       </c>
       <c r="D716" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in E minor</v>
       </c>
       <c r="E716" s="5" t="s">
@@ -25710,7 +25995,7 @@
         <v>1840</v>
       </c>
       <c r="D717" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in E-flat major</v>
       </c>
       <c r="E717" s="5" t="s">
@@ -25734,7 +26019,7 @@
         <v>1843</v>
       </c>
       <c r="D718" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in F major</v>
       </c>
       <c r="E718" s="5" t="s">
@@ -25758,7 +26043,7 @@
         <v>1845</v>
       </c>
       <c r="D719" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in F major</v>
       </c>
       <c r="E719" s="5" t="s">
@@ -25782,7 +26067,7 @@
         <v>1848</v>
       </c>
       <c r="D720" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in F major</v>
       </c>
       <c r="E720" s="5" t="s">
@@ -25806,7 +26091,7 @@
         <v>1850</v>
       </c>
       <c r="D721" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in F major</v>
       </c>
       <c r="E721" s="5" t="s">
@@ -25830,7 +26115,7 @@
         <v>1852</v>
       </c>
       <c r="D722" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in G major</v>
       </c>
       <c r="E722" s="5" t="s">
@@ -25854,7 +26139,7 @@
         <v>1854</v>
       </c>
       <c r="D723" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in G major</v>
       </c>
       <c r="E723" s="5" t="s">
@@ -25878,7 +26163,7 @@
         <v>1856</v>
       </c>
       <c r="D724" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in G major</v>
       </c>
       <c r="E724" s="5" t="s">
@@ -25899,7 +26184,7 @@
         <v>1217</v>
       </c>
       <c r="D725" s="4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="17"/>
         <v>Symphony in G major</v>
       </c>
       <c r="E725" s="5" t="s">
@@ -30658,7 +30943,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="B1:C1 E1:I1 B1031:C1125 E1031:I1125" numberStoredAsText="1"/>
+    <ignoredError sqref="E1031:I1125 B1031:C1125 E1:I1 B1:C1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>